<commit_message>
feat: halve EIM construction pts below booth mins
</commit_message>
<xml_diff>
--- a/data/xlsx/baci--electrical-installation-and-maintenance-construction.xlsx
+++ b/data/xlsx/baci--electrical-installation-and-maintenance-construction.xlsx
@@ -497,7 +497,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G42"/>
+  <dimension ref="A1:G43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15.17" customWidth="1" min="1" max="1"/>
@@ -1243,13 +1243,21 @@
         </is>
       </c>
     </row>
+    <row r="43" ht="28.3" customHeight="1">
+      <c r="A43" s="5" t="inlineStr">
+        <is>
+          <t>* For this course, the institute should have at least 15 channel wiring boards/booths and 3 concealed wiring booths. Otherwise, the total points achieved will be halved.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A13:G13"/>
     <mergeCell ref="C7:G7"/>
     <mergeCell ref="A1:G1"/>
     <mergeCell ref="A42:E42"/>
     <mergeCell ref="A39:D39"/>
+    <mergeCell ref="A43:G43"/>
     <mergeCell ref="A41:G41"/>
     <mergeCell ref="C8:G8"/>
     <mergeCell ref="A40:E40"/>

</xml_diff>